<commit_message>
Day 1 AI lesson and local changes
</commit_message>
<xml_diff>
--- a/GitHubRepository/00-Roadmaps/DailyChecklist/Daily_AI_Learning_Checklist_Template.xlsx
+++ b/GitHubRepository/00-Roadmaps/DailyChecklist/Daily_AI_Learning_Checklist_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dca33f22441cef85/Desktop/GitHubRepository/00-Roadmaps/DailyChecklist/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dca33f22441cef85/Documents/AI-Solution-Architect/GitHubRepository/00-Roadmaps/DailyChecklist/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F2E45E0-22A0-4530-AD97-DC459573E615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{0F2E45E0-22A0-4530-AD97-DC459573E615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACA90782-F097-48BA-9A79-18A54EFD48DC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>AI Solution Architect - Daily Learning Checklist</t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>Overall Self Rating (1-10)</t>
+  </si>
+  <si>
+    <t>The Foundation of Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>1 hour</t>
   </si>
 </sst>
 </file>
@@ -184,13 +190,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,7 +505,7 @@
   <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
@@ -506,268 +515,289 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
+      <c r="B3" s="7">
+        <v>46236</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
+      <c r="B4" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
+      <c r="B5" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="6" t="s">
         <v>4</v>
       </c>
+      <c r="B6" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
+      <c r="B7" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
+      <c r="B8" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
+      <c r="B9" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="5">
+      <c r="A12" s="3">
         <v>1</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="5">
+      <c r="A13" s="3">
         <v>2</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="5">
+      <c r="A14" s="3">
         <v>3</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="5">
+      <c r="A15" s="3">
         <v>4</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="5">
+      <c r="A16" s="3">
         <v>5</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="5">
+      <c r="A17" s="3">
         <v>6</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="5">
+      <c r="A18" s="3">
         <v>7</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="5">
+      <c r="A19" s="3">
         <v>8</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="5">
+      <c r="A20" s="3">
         <v>9</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="5">
+      <c r="A21" s="3">
         <v>10</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="5">
+      <c r="A22" s="3">
         <v>11</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="5">
+      <c r="A23" s="3">
         <v>12</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="5">
+      <c r="A24" s="3">
         <v>13</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="5">
+      <c r="A25" s="3">
         <v>14</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="5">
+      <c r="A26" s="3">
         <v>15</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">

</xml_diff>